<commit_message>
Rebin Keynote line series to standard round price anchors
Replace geometric-midpoint x labels (0.12, 0.19, ...) with round anchor
prices ($0.5, $1, $2, $5, $10, $20, $50, $100); each card assigned to its
nearest anchor. Easier to read as chart axis labels.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/keynote_chart_data.xlsx
+++ b/output/keynote_chart_data.xlsx
@@ -425,10 +425,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -437,7 +437,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Price ($, log)</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -457,241 +457,131 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>0.12</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>$0.5</t>
+        </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>159.6</v>
+        <v>63</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>11.2</v>
+        <v>-46</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>8</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>0.19</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>$1</t>
+        </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-25</v>
+        <v>-53</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>41</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>0.29</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>$2</t>
+        </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45.8</v>
+        <v>34</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-48.3</v>
+        <v>-29</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>0.44</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>$5</t>
+        </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>59.6</v>
+        <v>37</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-58.9</v>
+        <v>-11</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>86</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>0.68</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>61.2</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-50.5</v>
+        <v>-8</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>38</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>1.04</v>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>$20</t>
+        </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45.7</v>
+        <v>17</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-57.4</v>
+        <v>-5</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>48</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>1.59</v>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>$50</t>
+        </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>38.2</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-37.9</v>
+        <v>-4</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>2.44</v>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>36.2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-27.3</v>
+        <v>-19</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>-12.6</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>34.4</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>-9.4</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>13.39</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>-8</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>-5</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>31.39</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>-3.2</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>48.06</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>73.56999999999999</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>-15.7</v>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>112.63</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>-18.7</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Extend Keynote line series to a $200 anchor
Add $200 price bucket to the round-anchor line series (x now
$0.5..$200). Note: $100 and $200 buckets are thin (8 and 5 cards).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/keynote_chart_data.xlsx
+++ b/output/keynote_chart_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -575,13 +575,29 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>-19</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>13</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>$200</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>-11</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>